<commit_message>
data update + bibliography
</commit_message>
<xml_diff>
--- a/raw/Feature_lists.xlsx
+++ b/raw/Feature_lists.xlsx
@@ -9,7 +9,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>id</t>
   </si>
@@ -20,10 +20,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>authors</t>
-  </si>
-  <si>
-    <t>number of features</t>
+    <t>description</t>
   </si>
   <si>
     <t>year</t>
@@ -32,6 +29,12 @@
     <t>SAILS</t>
   </si>
   <si>
+    <t>https://sails.clld.org/</t>
+  </si>
+  <si>
+    <t>Pieter Muysken, Harald Hammarström, Olga Krasnoukhova, Neele Müller, Joshua Birchall, Simon van de Kerke, Loretta O'Connor, Swintha Danielsen, Rik van Gijn &amp; George Saad</t>
+  </si>
+  <si>
     <t>WALS</t>
   </si>
   <si>
@@ -47,7 +50,7 @@
     <t>http://grambank.clld.org/</t>
   </si>
   <si>
-    <t>Harald Hammarström, Hedvig Skirgård, et al.</t>
+    <t>Hedvig Skirgård et al.</t>
   </si>
   <si>
     <t>SSWL</t>
@@ -81,13 +84,22 @@
   </si>
   <si>
     <t>Susanne Michaelis, Philippe Maurer, Martin Haspelmath, Magnus Huber</t>
+  </si>
+  <si>
+    <t>ATLAs Zurich</t>
+  </si>
+  <si>
+    <t>https://atlas.evolvinglanguage.ch</t>
+  </si>
+  <si>
+    <t>David Inman et al.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="10">
+  <numFmts count="9">
     <numFmt formatCode="@" numFmtId="165"/>
     <numFmt formatCode="mm/dd/yyyy" numFmtId="166"/>
     <numFmt formatCode="[hh]:mm:ss" numFmtId="167"/>
@@ -129,7 +141,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0"/>
     <xf applyAlignment="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -154,9 +166,6 @@
       <alignment horizontal="general" vertical="top"/>
     </xf>
     <xf applyAlignment="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="171" xfId="0">
-      <alignment horizontal="general" vertical="top"/>
-    </xf>
-    <xf applyAlignment="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0">
       <alignment horizontal="general" vertical="top"/>
     </xf>
     <xf applyAlignment="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0">
@@ -186,16 +195,22 @@
       <c r="E1" t="s" s="1">
         <v>4</v>
       </c>
-      <c r="F1" t="s" s="1">
-        <v>5</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="6">
         <v>2</v>
       </c>
       <c r="B2" t="s" s="7">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s" s="8">
         <v>6</v>
+      </c>
+      <c r="D2" t="s" s="9">
+        <v>7</v>
+      </c>
+      <c r="E2" s="10">
+        <v>2016</v>
       </c>
     </row>
     <row r="3">
@@ -203,18 +218,15 @@
         <v>3</v>
       </c>
       <c r="B3" t="s" s="7">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s" s="8">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D3" t="s" s="9">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E3" s="10">
-        <v>192</v>
-      </c>
-      <c r="F3" s="11">
         <v>2013</v>
       </c>
     </row>
@@ -223,19 +235,16 @@
         <v>4</v>
       </c>
       <c r="B4" t="s" s="7">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C4" t="s" s="8">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D4" t="s" s="9">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E4" s="10">
-        <v>195</v>
-      </c>
-      <c r="F4" s="11">
-        <v>2015</v>
+        <v>2023</v>
       </c>
     </row>
     <row r="5">
@@ -243,10 +252,10 @@
         <v>5</v>
       </c>
       <c r="B5" t="s" s="7">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C5" t="s" s="8">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6">
@@ -254,18 +263,15 @@
         <v>6</v>
       </c>
       <c r="B6" t="s" s="7">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C6" t="s" s="8">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D6" t="s" s="9">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E6" s="10">
-        <v>304</v>
-      </c>
-      <c r="F6" s="11">
         <v>0</v>
       </c>
     </row>
@@ -274,15 +280,15 @@
         <v>7</v>
       </c>
       <c r="B7" t="s" s="7">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C7" t="s" s="8">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D7" t="s" s="9">
-        <v>20</v>
-      </c>
-      <c r="F7" s="11">
+        <v>21</v>
+      </c>
+      <c r="E7" s="10">
         <v>2017</v>
       </c>
     </row>
@@ -291,16 +297,33 @@
         <v>1</v>
       </c>
       <c r="B8" t="s" s="7">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C8" t="s" s="8">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D8" t="s" s="9">
-        <v>23</v>
-      </c>
-      <c r="F8" s="11">
+        <v>24</v>
+      </c>
+      <c r="E8" s="10">
         <v>2013</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s" s="7">
+        <v>25</v>
+      </c>
+      <c r="C9" t="s" s="8">
+        <v>26</v>
+      </c>
+      <c r="D9" t="s" s="9">
+        <v>27</v>
+      </c>
+      <c r="E9" s="10">
+        <v>2025</v>
       </c>
     </row>
   </sheetData>

</xml_diff>